<commit_message>
feat(wietnauer-v3): Sprint 2 — rapor yapısı Top8+Diğer, KPI Hacim, foresight isim (Faz 1)
- md6: KPI şeridi Hacim ilk sıra (Toplam Hacim 70cl) + Net Ciro
- md17: Cockpit heatmap Top6 -> Top8 + Diğer (JOIN+ISNULL; 9 sütun)
- md18: Portföy Top10 -> Top8 + Diğer (UNION ALL; 9 satır)
- md29/30/36/37: Marka Portföy/TopSKU/Penetrasyon Diğer + dip toplam
- md13: Foresight alanlarına anlaşılır Türkçe isimler
- foldOther + sumBy ortak yardımcısı (gizlenen kalem 'Diğer'de görünsün)
- eforlama.xlsx: 'Yapılan İşler' sheet
</commit_message>
<xml_diff>
--- a/docs/weitnauer-v3-eforlama.xlsx
+++ b/docs/weitnauer-v3-eforlama.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Planı" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talepler" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yapılan İşler" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Planı" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talepler" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Talepler'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Talepler'!$A$1:$I$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,8 +131,27 @@
       <color rgb="00B00020"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B7A3D"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -158,8 +178,23 @@
         <fgColor rgb="00D6EFD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EEF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F4E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -181,11 +216,69 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -263,6 +356,23 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -629,6 +739,393 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Weitnauer v3 — Tamamlanan İşler (Hafta 1–2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>Faz 0 + Faz 1 (ilk 2 hafta) · 22 saat efor · kod tamamlandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Hafta</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>Madde</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>Yapılan iş</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>Durum</t>
+        </is>
+      </c>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>Doğrulama</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Hafta 1 — Doğruluk &amp; temizlik (Faz 0) · 11.5 saat · 🚀 Deploy #1 (canlıda)</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="n"/>
+      <c r="C5" s="34" t="n"/>
+      <c r="D5" s="34" t="n"/>
+      <c r="E5" s="35" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="inlineStr">
+        <is>
+          <t>md19</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Haritada pasif müşteri/dağıtıcı noktaları temizlendi (BYTDURUM=0 filtresi) + resync</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>23.873 → 11.942 nokta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>md33</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Segment ek grup bağlantısı m2m junction yerine direkt bağlantıya çevrildi</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>junction 0 satır → direkt 15.483 satır</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>md7</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>70cl Hacim formülü düzeltildi; divisor tenant-config e taşındı (wietnauer=1)</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>113.976 = 9 × 12.664 doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>"Diğer" + dip toplam ortak yardımcısı (foldOther + sumBy) yazıldı</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>packages/core/src/fold-other.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>md25/31/32/39/40</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Gereksiz panel ve kolonlar kaldırıldı</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 1</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>md8</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Doğrulama yapıldı</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Hafta 2 — Rapor yapısı (Faz 1) · 10.5 saat · 🚀 Deploy #2 (bekliyor)</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="n"/>
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="34" t="n"/>
+      <c r="E12" s="35" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 2</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>md6</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>KPI şeridi yeniden dizildi: ilk kart Toplam Hacim (70cl), ikinci Net Ciro</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>warm OK, hacim+ciro id korundu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 2</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>md17</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Cockpit heatmap Top 6 → Top 8 + Diğer (JOIN+ISNULL bucketing)</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>9 sütun doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 2</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>md18</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Portföy paneli Top 10 → Top 8 + Diğer (UNION ALL)</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>9 satır doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 2</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>md29/30/36/37</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Marka ekranı (Portföy / Top SKU / Penetrasyon) Diğer + dip toplam satırı</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="inlineStr">
+        <is>
+          <t>typecheck temiz, warm OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="36" t="inlineStr">
+        <is>
+          <t>Hafta 2</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>md13</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Foresight alanlarına anlaşılır Türkçe isimler</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A5:E5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -963,7 +1460,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3106,7 +3603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(wietnauer): panorama bilgi modeli + pusula branding + eforlama & yapılan-işler raporları
</commit_message>
<xml_diff>
--- a/docs/weitnauer-v3-eforlama.xlsx
+++ b/docs/weitnauer-v3-eforlama.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -149,6 +149,23 @@
     <font>
       <b val="1"/>
       <color rgb="001B7A3D"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E7D34"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="9">
@@ -278,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -372,6 +389,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -739,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -759,7 +788,7 @@
     <row r="2">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>Faz 0 + Faz 1 (ilk 2 hafta) · 22 saat efor · kod tamamlandı</t>
+          <t>Faz 0 + Faz 1 + Hafta 3 (metrik doğruluğu) + Kullanıcı Yetkilendirme &amp; Yönetim</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1138,298 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>Hafta 3 — Metrik Doğruluğu (Faz 1) · 4 madde</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>Hafta 3</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>md22</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>Yönetim: Top Müşteri analizi → Top Distribütör analizine çevrildi</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr">
+        <is>
+          <t>canlı doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>Hafta 3</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>md23</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>Top distribütör tablosuna aktif müşteri sayısı + FKMS/kapsama eklendi</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>aktif müşteri + FKMS sütunları</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>Hafta 3</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t>md26</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
+        <is>
+          <t>Birim TL↔Hacim değişince distribütör cirosu Hacim'e döner</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E21" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>Hafta 3</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="inlineStr">
+        <is>
+          <t>md41</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>Saha: temsilci müşteri kolonu → aktif müşteri sayısı</t>
+        </is>
+      </c>
+      <c r="D22" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>Kullanıcı Yetkilendirme &amp; Yönetim (ek geliştirme) · canlı doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>Kullanıcı yetkilendirme: hangi kullanıcı hangi ekranı görebilir tanımlanabiliyor</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>ekran erişimi + navbar filtresi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>Distribütör-bazlı veri erişimi: kullanıcı yalnızca Panorama'da yetkili olduğu distribütörleri görür</t>
+        </is>
+      </c>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>firat.das 2 dist / ERCYONETICI 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>Yalnızca merkez (BYTTIP=0) kullanıcı erişimi; distribütör hesapları giremez</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>login/scope/oturum 3 katman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>Yönetim paneli: ekran başlık/içerik + kullanıcı yetkileri panelden yönetilir</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
+        <is>
+          <t>içerik override + Yetkiler ekranı</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>Admin yetkisi devredilebilir (yönetici başka kullanıcıya yetki verebilir)</t>
+        </is>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>ERCYONETICI + verdikleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="inlineStr">
+        <is>
+          <t>Ek</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>Oturum güvenliği: oturum düştüğünde temiz giriş yönlendirmesi + navbar düzeltmesi</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>✅ Tamam</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>canlı test edildi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>